<commit_message>
Normalización del modelo relacional
</commit_message>
<xml_diff>
--- a/Segundo trimestre/Normalizacion ArteNauta.xlsx
+++ b/Segundo trimestre/Normalizacion ArteNauta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ea054\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{611AC825-8991-45C9-895D-BC88F01DABF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{141375DF-5D3F-49B1-B3E2-064908F755E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="240">
   <si>
     <t>Nombre_Admin</t>
   </si>
@@ -725,6 +725,24 @@
   </si>
   <si>
     <t>Ya queda como el modelo final: todas las tablas separadas (Usuario, Artista, Publicación, Comentario, etc.).</t>
+  </si>
+  <si>
+    <t>idSolicitud</t>
+  </si>
+  <si>
+    <t>fechaSolicitud</t>
+  </si>
+  <si>
+    <t>tipoSolicitud</t>
+  </si>
+  <si>
+    <t>estadoSolicitud</t>
+  </si>
+  <si>
+    <t>Verificado</t>
+  </si>
+  <si>
+    <t>En espera</t>
   </si>
 </sst>
 </file>
@@ -758,7 +776,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -776,8 +794,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9CE91"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -824,11 +848,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -857,7 +894,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -866,24 +903,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFA9CE91"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2018,19 +2073,15 @@
       </c>
     </row>
     <row r="15" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="C15" s="14"/>
       <c r="D15" s="11"/>
     </row>
     <row r="16" spans="2:27" x14ac:dyDescent="0.3">
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2080,7 +2131,7 @@
       <c r="H2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="13" t="s">
         <v>227</v>
       </c>
     </row>
@@ -2106,12 +2157,12 @@
       <c r="H3" s="1">
         <v>3159276217</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
@@ -2135,12 +2186,12 @@
       <c r="H4" s="1">
         <v>3118692159</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="15" t="s">
         <v>228</v>
       </c>
-      <c r="K4" s="12"/>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
@@ -2505,7 +2556,7 @@
       <c r="H2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="13" t="s">
         <v>227</v>
       </c>
     </row>
@@ -2531,12 +2582,12 @@
       <c r="H3" s="3">
         <v>45991</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
@@ -2560,15 +2611,15 @@
       <c r="H4" s="3">
         <v>45991</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
@@ -3256,7 +3307,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B2:P69"/>
+  <dimension ref="B2:P74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3293,7 +3344,7 @@
       <c r="H2" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="13" t="s">
         <v>227</v>
       </c>
     </row>
@@ -3319,15 +3370,15 @@
       <c r="H3" s="3">
         <v>45991</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="16" t="s">
         <v>233</v>
       </c>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="1">
@@ -3351,12 +3402,12 @@
       <c r="H4" s="3">
         <v>45991</v>
       </c>
-      <c r="J4" s="17" t="s">
+      <c r="J4" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" s="1">
@@ -3475,95 +3526,73 @@
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="C16" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>172</v>
+      <c r="D16" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B17" s="1">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="H17" s="3">
-        <v>45992</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="J17" s="1">
-        <v>3</v>
+      <c r="B17" s="20">
+        <v>1</v>
+      </c>
+      <c r="C17" s="20">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3">
+        <v>45996</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B18" s="1">
-        <v>2</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="H18" s="3">
-        <v>45993</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="J18" s="1">
-        <v>4</v>
-      </c>
+      <c r="B18" s="19">
+        <v>2</v>
+      </c>
+      <c r="C18" s="19">
+        <v>2</v>
+      </c>
+      <c r="D18" s="3">
+        <v>45996</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B21" s="2" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>155</v>
@@ -3572,7 +3601,7 @@
         <v>156</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>158</v>
@@ -3581,159 +3610,189 @@
         <v>159</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="K21" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="22" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B22" s="1">
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J22" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="H22" s="3">
+        <v>45992</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="K22" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J22" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B23" s="1">
         <v>2</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="K23" s="1">
-        <v>2</v>
+        <v>174</v>
+      </c>
+      <c r="H23" s="3">
+        <v>45993</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="J23" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B26" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>182</v>
+        <v>155</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.3">
+        <v>156</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B27" s="1">
         <v>1</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="K27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B28" s="1">
         <v>2</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>185</v>
+        <v>56</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B31" s="2" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>191</v>
-      </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <v>1</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="E32" s="3">
-        <v>45200</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G32" s="1">
-        <v>1</v>
-      </c>
-      <c r="H32" s="1">
-        <v>1</v>
+        <v>184</v>
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.3">
@@ -3741,98 +3800,113 @@
         <v>2</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="E33" s="3">
-        <v>45235</v>
-      </c>
-      <c r="F33" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B36" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B37" s="1">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" s="3">
+        <v>45200</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="G33" s="1">
-        <v>2</v>
-      </c>
-      <c r="H33" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B34" s="1">
-        <v>3</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E34" s="3">
-        <v>45270</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G34" s="1">
-        <v>1</v>
-      </c>
-      <c r="H34" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B37" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>195</v>
+      <c r="G37" s="1">
+        <v>1</v>
+      </c>
+      <c r="H37" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B38" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D38" s="3">
-        <v>45200</v>
-      </c>
-      <c r="E38" s="1">
-        <v>1</v>
+        <v>61</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E38" s="3">
+        <v>45235</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G38" s="1">
+        <v>2</v>
+      </c>
+      <c r="H38" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B39" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D39" s="3">
-        <v>45236</v>
-      </c>
-      <c r="E39" s="1">
-        <v>2</v>
+        <v>134</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E39" s="3">
+        <v>45270</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G39" s="1">
+        <v>1</v>
+      </c>
+      <c r="H39" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B42" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>195</v>
@@ -3842,11 +3916,11 @@
       <c r="B43" s="1">
         <v>1</v>
       </c>
-      <c r="C43" s="3">
+      <c r="C43" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D43" s="3">
         <v>45200</v>
-      </c>
-      <c r="D43" s="1">
-        <v>1</v>
       </c>
       <c r="E43" s="1">
         <v>1</v>
@@ -3856,11 +3930,11 @@
       <c r="B44" s="1">
         <v>2</v>
       </c>
-      <c r="C44" s="3">
+      <c r="C44" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D44" s="3">
         <v>45236</v>
-      </c>
-      <c r="D44" s="1">
-        <v>2</v>
       </c>
       <c r="E44" s="1">
         <v>2</v>
@@ -3868,23 +3942,29 @@
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B47" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B48" s="1">
         <v>1</v>
       </c>
-      <c r="C48" s="1" t="s">
-        <v>84</v>
+      <c r="C48" s="3">
+        <v>45200</v>
       </c>
       <c r="D48" s="1">
+        <v>1</v>
+      </c>
+      <c r="E48" s="1">
         <v>1</v>
       </c>
     </row>
@@ -3892,114 +3972,96 @@
       <c r="B49" s="1">
         <v>2</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="3">
+        <v>45236</v>
+      </c>
+      <c r="D49" s="1">
+        <v>2</v>
+      </c>
+      <c r="E49" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B52" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B53" s="1">
+        <v>1</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D53" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B54" s="1">
+        <v>2</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D49" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B50" s="1">
-        <v>3</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D50" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B51" s="1">
-        <v>4</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D51" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B54" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>205</v>
+      <c r="D54" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B55" s="1">
-        <v>1</v>
-      </c>
-      <c r="C55" s="3">
-        <v>45231</v>
+        <v>3</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>84</v>
       </c>
       <c r="D55" s="1">
-        <v>1</v>
-      </c>
-      <c r="E55" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B56" s="1">
-        <v>2</v>
-      </c>
-      <c r="C56" s="3">
-        <v>45250</v>
+        <v>4</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="D56" s="1">
-        <v>3</v>
-      </c>
-      <c r="E56" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B59" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>144</v>
+        <v>204</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B60" s="1">
         <v>1</v>
       </c>
-      <c r="C60" s="1">
-        <v>1</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E60" s="3">
+      <c r="C60" s="3">
         <v>45231</v>
       </c>
-      <c r="F60" s="1">
-        <v>1</v>
-      </c>
-      <c r="G60" s="1">
+      <c r="D60" s="1">
+        <v>1</v>
+      </c>
+      <c r="E60" s="1">
         <v>2</v>
       </c>
     </row>
@@ -4007,151 +4069,205 @@
       <c r="B61" s="1">
         <v>2</v>
       </c>
-      <c r="C61" s="1">
-        <v>1</v>
-      </c>
-      <c r="D61" s="4" t="s">
+      <c r="C61" s="3">
+        <v>45250</v>
+      </c>
+      <c r="D61" s="1">
+        <v>3</v>
+      </c>
+      <c r="E61" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B64" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="65" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B65" s="1">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1">
+        <v>1</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E65" s="3">
+        <v>45231</v>
+      </c>
+      <c r="F65" s="1">
+        <v>1</v>
+      </c>
+      <c r="G65" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B66" s="1">
+        <v>2</v>
+      </c>
+      <c r="C66" s="1">
+        <v>1</v>
+      </c>
+      <c r="D66" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E61" s="3">
+      <c r="E66" s="3">
         <v>45231</v>
       </c>
-      <c r="F61" s="1">
-        <v>2</v>
-      </c>
-      <c r="G61" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B62" s="1">
-        <v>3</v>
-      </c>
-      <c r="C62" s="1">
-        <v>2</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E62" s="3">
-        <v>45250</v>
-      </c>
-      <c r="F62" s="1">
-        <v>3</v>
-      </c>
-      <c r="G62" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="63" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B63" s="1">
-        <v>4</v>
-      </c>
-      <c r="C63" s="1">
-        <v>2</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E63" s="3">
-        <v>45250</v>
-      </c>
-      <c r="F63" s="1">
-        <v>4</v>
-      </c>
-      <c r="G63" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="66" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B66" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>198</v>
+      <c r="F66" s="1">
+        <v>2</v>
+      </c>
+      <c r="G66" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B67" s="1">
-        <v>1</v>
-      </c>
-      <c r="C67" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C67" s="1">
+        <v>2</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E67" s="3">
+        <v>45250</v>
+      </c>
+      <c r="F67" s="1">
+        <v>3</v>
+      </c>
+      <c r="G67" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B68" s="1">
+        <v>4</v>
+      </c>
+      <c r="C68" s="1">
+        <v>2</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E68" s="3">
+        <v>45250</v>
+      </c>
+      <c r="F68" s="1">
+        <v>4</v>
+      </c>
+      <c r="G68" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B71" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B72" s="1">
+        <v>1</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D67" s="1" t="s">
+      <c r="D72" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="E67" s="3">
+      <c r="E72" s="3">
         <v>45992</v>
       </c>
-      <c r="F67" s="1">
-        <v>1</v>
-      </c>
-      <c r="G67" s="1">
-        <v>1</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B68" s="1">
-        <v>2</v>
-      </c>
-      <c r="C68" s="1" t="s">
+      <c r="F72" s="1">
+        <v>1</v>
+      </c>
+      <c r="G72" s="1">
+        <v>1</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="73" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B73" s="1">
+        <v>2</v>
+      </c>
+      <c r="C73" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D68" s="1" t="s">
+      <c r="D73" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E68" s="3">
+      <c r="E73" s="3">
         <v>45992</v>
       </c>
-      <c r="F68" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="G68" s="1">
-        <v>2</v>
-      </c>
-      <c r="H68" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B69" s="1">
+      <c r="F73" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G73" s="1">
+        <v>2</v>
+      </c>
+      <c r="H73" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B74" s="1">
         <v>3</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C74" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D69" s="1" t="s">
+      <c r="D74" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E69" s="3">
+      <c r="E74" s="3">
         <v>45993</v>
       </c>
-      <c r="F69" s="1">
-        <v>2</v>
-      </c>
-      <c r="G69" s="1">
+      <c r="F74" s="1">
+        <v>2</v>
+      </c>
+      <c r="G74" s="1">
         <v>3</v>
       </c>
-      <c r="H69" s="1" t="s">
+      <c r="H74" s="1" t="s">
         <v>215</v>
       </c>
     </row>

</xml_diff>